<commit_message>
small change to available pipelines connections
</commit_message>
<xml_diff>
--- a/southern_europe/italy_data/network_capex_metrics/pipeline_size_class_connections.xlsx
+++ b/southern_europe/italy_data/network_capex_metrics/pipeline_size_class_connections.xlsx
@@ -2252,7 +2252,7 @@
         <v>1</v>
       </c>
       <c r="O14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P14" t="n">
         <v>1</v>
@@ -3786,7 +3786,7 @@
         <v>1</v>
       </c>
       <c r="X25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y25" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
removed some small connections
</commit_message>
<xml_diff>
--- a/southern_europe/italy_data/network_capex_metrics/pipeline_size_class_connections.xlsx
+++ b/southern_europe/italy_data/network_capex_metrics/pipeline_size_class_connections.xlsx
@@ -10102,7 +10102,7 @@
         <v>1</v>
       </c>
       <c r="Y26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z26" t="n">
         <v>1</v>
@@ -10111,7 +10111,7 @@
         <v>1</v>
       </c>
       <c r="AB26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC26" t="n">
         <v>1</v>
@@ -11377,7 +11377,7 @@
         <v>1</v>
       </c>
       <c r="AM35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN35" t="n">
         <v>1</v>

</xml_diff>